<commit_message>
write reporting log files
</commit_message>
<xml_diff>
--- a/trapper_data_report.xlsx
+++ b/trapper_data_report.xlsx
@@ -33746,7 +33746,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P106"/>
+  <dimension ref="A1:P107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -37873,6 +37873,52 @@
         </is>
       </c>
     </row>
+    <row r="107">
+      <c r="A107" s="2" t="inlineStr">
+        <is>
+          <t>FISHER</t>
+        </is>
+      </c>
+      <c r="B107" s="3" t="n">
+        <v>46314</v>
+      </c>
+      <c r="C107" s="2" t="n">
+        <v>49.34398918282288</v>
+      </c>
+      <c r="D107" s="2" t="n">
+        <v>-117.8696802434824</v>
+      </c>
+      <c r="E107" s="2" t="inlineStr"/>
+      <c r="F107" s="2" t="inlineStr">
+        <is>
+          <t>Not Reviewed</t>
+        </is>
+      </c>
+      <c r="G107" s="2" t="inlineStr"/>
+      <c r="H107" s="2" t="inlineStr"/>
+      <c r="I107" s="2" t="inlineStr"/>
+      <c r="J107" s="2" t="inlineStr">
+        <is>
+          <t>&lt;a href="mailto:?subject=Fisher Observation Response Summary&amp;body=Species: FISHER%0D%A0When did you see the fisher? 2026-10-19%0D%A0Observation Type: VISUAL%0D%A0Where did you see the fisher? (lat, long): 49.34398918282288 -117.86968024348238%0D%A0Photo Name: "&gt;Email me the response summary&lt;/a&gt;</t>
+        </is>
+      </c>
+      <c r="K107" s="4" t="n">
+        <v>46317.14858274306</v>
+      </c>
+      <c r="L107" s="2" t="inlineStr"/>
+      <c r="M107" s="2" t="inlineStr"/>
+      <c r="N107" s="2" t="inlineStr">
+        <is>
+          <t>VISUAL</t>
+        </is>
+      </c>
+      <c r="O107" s="2" t="inlineStr"/>
+      <c r="P107" s="2" t="inlineStr">
+        <is>
+          <t>&lt;100m</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>